<commit_message>
Member import: wedding date, household placement, customary marriages, no foreign instructions (Z1-Z4), tests first
The import reads Anniversary Date, places spouses and children in the main
person's sector and family group, treats customary and traditional
marriages as married (same rule as life phases), and the Import screen
lists its columns instead of another church's export script. Re-imported
the test file on the emulators: 34 records, all as expected.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/JCOC-Hub-Test-Members.xlsx
+++ b/docs/testing/JCOC-Hub-Test-Members.xlsx
@@ -3118,7 +3118,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E37"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -3152,7 +3152,7 @@
         <v>Thabo Nkosi</v>
       </c>
       <c r="C2" t="str">
-        <v>Parents of Kids &lt;10 (Young Married missing: import drops the wedding date)</v>
+        <v>Young Married, Parents of Kids &lt;10. Anniversary 2 December</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -3169,7 +3169,7 @@
         <v>Naledi Nkosi</v>
       </c>
       <c r="C3" t="str">
-        <v>Parents of Kids &lt;10 (Young Married missing, as above)</v>
+        <v>Young Married, Parents of Kids &lt;10. Same sector and family group as Thabo</v>
       </c>
       <c r="D3" t="str">
         <v/>
@@ -3220,7 +3220,7 @@
         <v>Pieter van Wyk</v>
       </c>
       <c r="C6" t="str">
-        <v>Parents of Kids &lt;&gt;10, Teen Parent (Mature Married missing: wedding date)</v>
+        <v>Mature Married, Parents of Kids &lt;&gt;10, Teen Parent</v>
       </c>
       <c r="D6" t="str">
         <v/>
@@ -3237,7 +3237,7 @@
         <v>Annelie van Wyk</v>
       </c>
       <c r="C7" t="str">
-        <v>Parents of Kids &lt;&gt;10, Teen Parent</v>
+        <v>Mature Married, Parents of Kids &lt;&gt;10, Teen Parent</v>
       </c>
       <c r="D7" t="str">
         <v/>
@@ -3407,7 +3407,7 @@
         <v>George Mahlangu</v>
       </c>
       <c r="C17" t="str">
-        <v>Empty Nester (Mature Married missing: wedding date)</v>
+        <v>Mature Married, Empty Nester. Anniversary 30 June</v>
       </c>
       <c r="D17" t="str">
         <v/>
@@ -3424,7 +3424,7 @@
         <v>Grace Mahlangu</v>
       </c>
       <c r="C18" t="str">
-        <v>Empty Nester</v>
+        <v>Mature Married, Empty Nester</v>
       </c>
       <c r="D18" t="str">
         <v/>
@@ -3509,7 +3509,7 @@
         <v>Ahmed Hassan</v>
       </c>
       <c r="C23" t="str">
-        <v>No phase (Mature Married missing: wedding date). Fatima is not in the member list; she is stored on the household as a non-member spouse</v>
+        <v>Mature Married. Fatima is not in the member list; she is stored on the household as a non-member spouse</v>
       </c>
       <c r="D23" t="str">
         <v/>
@@ -3560,7 +3560,7 @@
         <v>Mpho Sithole</v>
       </c>
       <c r="C26" t="str">
-        <v>Imported. Expect a problem: Palesa is NOT created, because the import only creates a spouse when the status is exactly 'Married'. Report this</v>
+        <v>Married (Customary) kept as written. Mature Married (married 2020, more than 5 years ago)</v>
       </c>
       <c r="D26" t="str">
         <v/>
@@ -3571,13 +3571,13 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>H13</v>
+        <v>H12</v>
       </c>
       <c r="B27" t="str">
-        <v>Nomsa Ndlovu</v>
+        <v>Palesa Sithole</v>
       </c>
       <c r="C27" t="str">
-        <v>Parents of Kids &gt;10 only. 'Separated' has no adult phase in the agreed list</v>
+        <v>Created as his spouse and linked to him, same sector and family group. Mature Married</v>
       </c>
       <c r="D27" t="str">
         <v/>
@@ -3591,10 +3591,10 @@
         <v>H13</v>
       </c>
       <c r="B28" t="str">
-        <v>Thando Ndlovu</v>
+        <v>Nomsa Ndlovu</v>
       </c>
       <c r="C28" t="str">
-        <v>Campus Student</v>
+        <v>Parents of Kids &gt;10 only. 'Separated' has no adult phase in the agreed list</v>
       </c>
       <c r="D28" t="str">
         <v/>
@@ -3605,13 +3605,13 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>H14</v>
+        <v>H13</v>
       </c>
       <c r="B29" t="str">
-        <v>Karabo Mokoena</v>
+        <v>Thando Ndlovu</v>
       </c>
       <c r="C29" t="str">
-        <v>Campus Student (anyone up to 20 counts as dependant age). Young Single starts at 21. Check this is what JCOC wants</v>
+        <v>Campus Student</v>
       </c>
       <c r="D29" t="str">
         <v/>
@@ -3622,13 +3622,13 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>H15</v>
+        <v>H14</v>
       </c>
       <c r="B30" t="str">
-        <v>Ruth Adams</v>
+        <v>Karabo Mokoena</v>
       </c>
       <c r="C30" t="str">
-        <v>Mature Single. Sector filled (Test sector), family group left blank for an admin to place</v>
+        <v>Campus Student (anyone up to 20 counts as dependant age). Young Single starts at 21. Check this is what JCOC wants</v>
       </c>
       <c r="D30" t="str">
         <v/>
@@ -3639,13 +3639,13 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>H16</v>
+        <v>H15</v>
       </c>
       <c r="B31" t="str">
-        <v>Peter Mensah</v>
+        <v>Ruth Adams</v>
       </c>
       <c r="C31" t="str">
-        <v>Mature Single. Sector and family group blank</v>
+        <v>Mature Single. Sector filled (Test sector), family group left blank for an admin to place</v>
       </c>
       <c r="D31" t="str">
         <v/>
@@ -3656,13 +3656,13 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>H17</v>
+        <v>H16</v>
       </c>
       <c r="B32" t="str">
-        <v>Yusuf Ebrahim</v>
+        <v>Peter Mensah</v>
       </c>
       <c r="C32" t="str">
-        <v>Born 15 August 1979, phone shown as 27825550190. Parents of Kids &gt;10, Teen Parent</v>
+        <v>Mature Single. Sector and family group blank</v>
       </c>
       <c r="D32" t="str">
         <v/>
@@ -3676,10 +3676,10 @@
         <v>H17</v>
       </c>
       <c r="B33" t="str">
-        <v>Ayesha Ebrahim</v>
+        <v>Yusuf Ebrahim</v>
       </c>
       <c r="C33" t="str">
-        <v>Born 12 September 1981, phone 27825550191. Parents of Kids &gt;10, Teen Parent</v>
+        <v>Born 15 August 1979, phone shown as 27825550190, anniversary 10 March 2005. Mature Married, Parents of Kids &gt;10, Teen Parent</v>
       </c>
       <c r="D33" t="str">
         <v/>
@@ -3693,10 +3693,10 @@
         <v>H17</v>
       </c>
       <c r="B34" t="str">
-        <v>Zaid Ebrahim</v>
+        <v>Ayesha Ebrahim</v>
       </c>
       <c r="C34" t="str">
-        <v>Teen, Scholar</v>
+        <v>Born 12 September 1981, phone 27825550191. Mature Married, Parents of Kids &gt;10, Teen Parent</v>
       </c>
       <c r="D34" t="str">
         <v/>
@@ -3707,13 +3707,13 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>H18</v>
+        <v>H17</v>
       </c>
       <c r="B35" t="str">
-        <v>Precious Mabaso</v>
+        <v>Zaid Ebrahim</v>
       </c>
       <c r="C35" t="str">
-        <v>Mature Single, Parents of Kids &lt;10. Add Single Mom by hand</v>
+        <v>Teen, Scholar</v>
       </c>
       <c r="D35" t="str">
         <v/>
@@ -3727,28 +3727,45 @@
         <v>H18</v>
       </c>
       <c r="B36" t="str">
+        <v>Precious Mabaso</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Mature Single, Parents of Kids &lt;10. Add Single Mom by hand</v>
+      </c>
+      <c r="D36" t="str">
+        <v/>
+      </c>
+      <c r="E36" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>H18</v>
+      </c>
+      <c r="B37" t="str">
         <v>Junior Mabaso</v>
       </c>
-      <c r="C36" t="str">
+      <c r="C37" t="str">
         <v>Child, Pre-School, Kidz Zone</v>
       </c>
-      <c r="D36" t="str">
-        <v/>
-      </c>
-      <c r="E36" t="str">
+      <c r="D37" t="str">
+        <v/>
+      </c>
+      <c r="E37" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E37"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A21"/>
   <cols>
     <col min="1" max="1" width="130.83203125" customWidth="1"/>
   </cols>
@@ -3800,7 +3817,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>4. The app should say 33 member records imported (18 households; non-member spouses and children are stored on households, not as members).</v>
+        <v>4. The app should say 34 member records imported (18 households; non-member spouses and children are stored on households, not as members).</v>
       </c>
     </row>
     <row r="11">
@@ -3810,7 +3827,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v xml:space="preserve">   Spouses and children will have no sector or family group (a known gap, below).</v>
+        <v xml:space="preserve">   Spouses and children are placed in the same sector and family group as the main person on their row.</v>
       </c>
     </row>
     <row r="13">
@@ -3835,42 +3852,32 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Known gaps this file is designed to show (report them, they are expected):</v>
+        <v>Things to know (expected behaviour, not faults):</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v xml:space="preserve">   - The import does not read the Anniversary Date column, so married people get no Young Married or Mature Married phase, and do not show under anniversaries.</v>
+        <v xml:space="preserve">   - Married couples should also appear under Birthdays &amp; Anniversaries when their anniversary is near.</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v xml:space="preserve">   - A spouse is only created when the status is exactly 'Married'. 'Married (Customary)' (H12) loses the spouse.</v>
+        <v xml:space="preserve">   - Single Mom and Single Dad are never automatic; they are added by hand on the member.</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v xml:space="preserve">   - Single Mom and Single Dad are never automatic; they are added by hand on the member.</v>
+        <v xml:space="preserve">   - People in different rows cannot be linked to each other by the import (for example a grown child who has her own household).</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v xml:space="preserve">   - People in different rows cannot be linked to each other by the import (for example a grown child who has her own household).</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v xml:space="preserve">   - Only the main person on each row is put in the sector and family group. Spouses and children are left unplaced, so leaders do not see them until an admin places them.</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
         <v xml:space="preserve">   - A single 19-year-old (H14) is a Campus Student, not a Young Single (that starts at 21).</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A21"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>